<commit_message>
feat(template): cores na evolução (verde >0, vermelho <0, branco =0)
Formatação condicional nas três colunas de evolução (KOD/E-level/Shape) via
CellIsRule. Zera a CF herdada da fonte (desalinhada pelo delete_cols) antes de
aplicar. As cores aparecem no .xlsx baixado (não na prévia do Streamlit).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/comparativo.xlsx
+++ b/templates/comparativo.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="780" windowWidth="34200" windowHeight="21460" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comparativo" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_aplicabilidade" sheetId="2" state="hidden" r:id="rId2"/>
+    <sheet name="Comparativo" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="_aplicabilidade" sheetId="2" state="hidden" r:id="rId2"/>
   </sheets>
   <externalReferences>
-    <externalReference xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+    <externalReference r:id="rId3"/>
   </externalReferences>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Comparativo'!$A$2:$H$134</definedName>
@@ -518,7 +518,7 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="4">
+  <dxfs count="7">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -553,6 +553,27 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00C6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFFFFF"/>
         </patternFill>
       </fill>
     </dxf>
@@ -630,8 +651,8 @@
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+<externalLink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <externalBook r:id="rId1">
     <sheetNames>
       <sheetName val="Original"/>
       <sheetName val="Comparativo"/>
@@ -16886,17 +16907,36 @@
     <mergeCell ref="F1:G1"/>
     <mergeCell ref="A1:A2"/>
   </mergeCells>
-  <conditionalFormatting sqref="A131">
-    <cfRule type="duplicateValues" priority="1" dxfId="3"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I3:I134 L3:L134">
-    <cfRule type="cellIs" priority="2" operator="lessThan" dxfId="2">
+  <conditionalFormatting sqref="E3:E134">
+    <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="4">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="greaterThan" dxfId="1">
+    <cfRule type="cellIs" priority="2" operator="lessThan" dxfId="5">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" dxfId="0">
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="6">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H3:H134">
+    <cfRule type="cellIs" priority="4" operator="greaterThan" dxfId="4">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="5" operator="lessThan" dxfId="5">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="6" operator="equal" dxfId="6">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K3:K134">
+    <cfRule type="cellIs" priority="7" operator="greaterThan" dxfId="4">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="8" operator="lessThan" dxfId="5">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="9" operator="equal" dxfId="6">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
fix(template): corrige cores da evolução e remove lixo da fonte
- Preenchimento da formatação condicional usava só fgColor com alpha 00
  (transparente e sem bgColor) -> Excel pedia "Repair" e não pintava. Passa
  a usar start/end_color em ARGB opaco (CF usa o bgColor).
- Remove as colunas à direita de "Evolução Shape" (realce amarelo de notas
  herdado da planilha-fonte).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/comparativo.xlsx
+++ b/templates/comparativo.xlsx
@@ -559,21 +559,24 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="00C6EFCE"/>
+          <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="00FFC7CE"/>
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="00FFFFFF"/>
+          <fgColor rgb="FFFFFFFF"/>
+          <bgColor rgb="FFFFFFFF"/>
         </patternFill>
       </fill>
     </dxf>
@@ -14491,7 +14494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L140"/>
+  <dimension ref="A1:K140"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="15" outlineLevelRow="1"/>
   <cols>
     <col outlineLevel="1" width="24.83203125" customWidth="1" style="4" min="1" max="1"/>
@@ -16118,7 +16121,6 @@
       <c r="I91" s="14" t="n"/>
       <c r="J91" s="15" t="n"/>
       <c r="K91" s="8" t="n"/>
-      <c r="L91" s="23" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="65" t="n"/>
@@ -16136,7 +16138,6 @@
       <c r="I92" s="14" t="n"/>
       <c r="J92" s="15" t="n"/>
       <c r="K92" s="8" t="n"/>
-      <c r="L92" s="23" t="n"/>
     </row>
     <row r="93" hidden="1" outlineLevel="1">
       <c r="A93" s="65" t="n"/>
@@ -16765,7 +16766,6 @@
       <c r="I128" s="14" t="n"/>
       <c r="J128" s="15" t="n"/>
       <c r="K128" s="42" t="n"/>
-      <c r="L128" s="23" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="65" t="n"/>
@@ -16783,7 +16783,6 @@
       <c r="I129" s="14" t="n"/>
       <c r="J129" s="15" t="n"/>
       <c r="K129" s="8" t="n"/>
-      <c r="L129" s="23" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="65" t="n"/>
@@ -16801,7 +16800,6 @@
       <c r="I130" s="14" t="n"/>
       <c r="J130" s="15" t="n"/>
       <c r="K130" s="8" t="n"/>
-      <c r="L130" s="23" t="n"/>
     </row>
     <row r="131">
       <c r="A131" s="65" t="n"/>
@@ -16819,7 +16817,6 @@
       <c r="I131" s="14" t="n"/>
       <c r="J131" s="15" t="n"/>
       <c r="K131" s="8" t="n"/>
-      <c r="L131" s="23" t="n"/>
     </row>
     <row r="132">
       <c r="A132" s="65" t="n"/>
@@ -16837,7 +16834,6 @@
       <c r="I132" s="14" t="n"/>
       <c r="J132" s="15" t="n"/>
       <c r="K132" s="8" t="n"/>
-      <c r="L132" s="23" t="n"/>
     </row>
     <row r="133">
       <c r="A133" s="66" t="n"/>
@@ -16855,7 +16851,6 @@
       <c r="I133" s="14" t="n"/>
       <c r="J133" s="15" t="n"/>
       <c r="K133" s="29" t="n"/>
-      <c r="L133" s="23" t="n"/>
     </row>
     <row r="134" ht="16" customHeight="1" thickBot="1">
       <c r="A134" s="45" t="inlineStr">

</xml_diff>

<commit_message>
fix(template): desloca larguras de coluna após remover a 1ª coluna
delete_cols não ajusta as larguras (mesmo caso de mesclagens/CF): a data de
Shape início caía numa coluna estreita e exibia "####", e o KOD herdava a
largura do Item. Cada coluna nova passa a herdar a largura da antiga c+1.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/comparativo.xlsx
+++ b/templates/comparativo.xlsx
@@ -14497,18 +14497,19 @@
   <dimension ref="A1:K140"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="15" outlineLevelRow="1"/>
   <cols>
-    <col outlineLevel="1" width="24.83203125" customWidth="1" style="4" min="1" max="1"/>
-    <col width="22.6640625" bestFit="1" customWidth="1" style="4" min="2" max="2"/>
-    <col width="47" customWidth="1" style="4" min="3" max="3"/>
-    <col hidden="1" outlineLevel="1" width="9.5" customWidth="1" style="4" min="4" max="4"/>
-    <col hidden="1" outlineLevel="1" width="10" customWidth="1" style="4" min="5" max="5"/>
-    <col hidden="1" outlineLevel="1" width="5.5" customWidth="1" style="4" min="6" max="6"/>
-    <col collapsed="1" width="9.6640625" bestFit="1" customWidth="1" style="4" min="7" max="7"/>
-    <col width="10" bestFit="1" customWidth="1" style="4" min="8" max="8"/>
-    <col width="8.5" customWidth="1" style="4" min="9" max="9"/>
-    <col width="9.6640625" bestFit="1" customWidth="1" style="4" min="10" max="10"/>
-    <col width="10" bestFit="1" customWidth="1" style="4" min="11" max="11"/>
-    <col width="9.1640625" customWidth="1" style="4" min="12" max="16384"/>
+    <col outlineLevel="1" width="22.6640625" customWidth="1" style="4" min="1" max="1"/>
+    <col width="47" bestFit="1" customWidth="1" style="4" min="2" max="2"/>
+    <col width="9.5" customWidth="1" style="4" min="3" max="3"/>
+    <col hidden="1" outlineLevel="1" width="10" customWidth="1" style="4" min="4" max="4"/>
+    <col hidden="1" outlineLevel="1" width="5.5" customWidth="1" style="4" min="5" max="5"/>
+    <col hidden="1" outlineLevel="1" width="9.6640625" customWidth="1" style="4" min="6" max="6"/>
+    <col collapsed="1" width="10" bestFit="1" customWidth="1" style="4" min="7" max="7"/>
+    <col width="8.5" bestFit="1" customWidth="1" style="4" min="8" max="8"/>
+    <col width="9.6640625" customWidth="1" style="4" min="9" max="9"/>
+    <col width="10" bestFit="1" customWidth="1" style="4" min="10" max="10"/>
+    <col width="9.1640625" bestFit="1" customWidth="1" style="4" min="11" max="11"/>
+    <col width="13" customWidth="1" style="4" min="12" max="16384"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>

<commit_message>
Propagate period dates into comparison headers
</commit_message>
<xml_diff>
--- a/templates/comparativo.xlsx
+++ b/templates/comparativo.xlsx
@@ -976,11 +976,11 @@
   <cols>
     <col outlineLevel="1" width="22.6640625" customWidth="1" style="4" min="1" max="1"/>
     <col width="47" bestFit="1" customWidth="1" style="4" min="2" max="2"/>
-    <col width="9.5" customWidth="1" style="4" min="3" max="3"/>
-    <col hidden="1" outlineLevel="1" width="10" customWidth="1" style="4" min="4" max="4"/>
-    <col hidden="1" outlineLevel="1" width="5.5" customWidth="1" style="4" min="5" max="5"/>
-    <col hidden="1" outlineLevel="1" width="9.6640625" customWidth="1" style="4" min="6" max="6"/>
-    <col collapsed="1" width="10" bestFit="1" customWidth="1" style="4" min="7" max="7"/>
+    <col width="9.5" customWidth="1" style="4" min="3" max="3" hidden="1"/>
+    <col hidden="1" width="10" customWidth="1" style="4" min="4" max="4"/>
+    <col hidden="1" width="5.5" customWidth="1" style="4" min="5" max="5"/>
+    <col width="9.6640625" customWidth="1" style="4" min="6" max="6"/>
+    <col width="10" bestFit="1" customWidth="1" style="4" min="7" max="7"/>
     <col width="8.5" bestFit="1" customWidth="1" style="4" min="8" max="8"/>
     <col width="9.6640625" customWidth="1" style="4" min="9" max="9"/>
     <col width="10" bestFit="1" customWidth="1" style="4" min="10" max="10"/>

</xml_diff>